<commit_message>
feat: cột Vị trí kệ — hiện 📍 trên thẻ thuốc và Tra thuốc, gõ mã kệ ra thuốc kệ đó (1.0.5)
</commit_message>
<xml_diff>
--- a/CatLieuNhanh_mau.xlsx
+++ b/CatLieuNhanh_mau.xlsx
@@ -15,7 +15,7 @@
     <sheet name="Danh mục" sheetId="6" state="hidden" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Thuốc'!$A$1:$I$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Thuốc'!$A$1:$J$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Luật cắt liều'!$A$1:$L$83</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Triệu chứng'!$A$1:$D$28</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Dấu hiệu nguy hiểm'!$A$1:$C$14</definedName>
@@ -260,6 +260,11 @@
     <comment ref="H1" authorId="0" shapeId="0">
       <text>
         <t>Ghi Có nếu là thuốc kê đơn (kháng sinh, corticoid...). App sẽ không tự gợi ý và nhắc hỏi dược sĩ.</t>
+      </text>
+    </comment>
+    <comment ref="I1" authorId="0" shapeId="0">
+      <text>
+        <t>Chỗ để thuốc ở quầy, ghi đúng nhãn dán trên kệ: Kệ A3, Ngăn kéo 2, Tủ lạnh... App in dưới tên thuốc để nhân viên mới tìm được. Gõ mã kệ ở tab Tra thuốc sẽ ra hết thuốc kệ đó.</t>
       </text>
     </comment>
   </commentList>
@@ -650,7 +655,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
+  <dimension ref="A1:A18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -707,53 +712,60 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Cột Còn hàng: Có / Hết. Thuốc khách hay hỏi mà quầy chưa nhập cũng ghi vào và đánh Hết → nhân viên tra được và app chỉ thuốc thay thế đang có. Cột Kê đơn: ghi Có với kháng sinh, corticoid... app sẽ không tự gợi ý.</t>
+          <t>Cột Vị trí: ghi đúng nhãn dán trên kệ (Kệ A3, Ngăn kéo 2, Tủ lạnh) để nhân viên mới tìm được thuốc. Nên dán nhãn kệ theo chữ+số rồi ghi y vậy.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Sheet Luật cắt liều: mỗi dòng = 1 triệu chứng + 1 đối tượng + 1 hoạt chất. Điền mg/kg/lần (app nhân số kg) HOẶC mg cố định/lần. Không tính theo mg thì viết vào Liều ghi tay.</t>
+          <t>Cột Còn hàng: Có / Hết. Thuốc khách hay hỏi mà quầy chưa nhập cũng ghi vào và đánh Hết → nhân viên tra được và app chỉ thuốc thay thế đang có. Cột Kê đơn: ghi Có với kháng sinh, corticoid... app sẽ không tự gợi ý.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Sheet Triệu chứng: xếp chip trên màn hình + cột 'Khách hay nói' để nhân viên gõ lời khách là ra chip đúng.</t>
+          <t>Sheet Luật cắt liều: mỗi dòng = 1 triệu chứng + 1 đối tượng + 1 hoạt chất. Điền mg/kg/lần (app nhân số kg) HOẶC mg cố định/lần. Không tính theo mg thì viết vào Liều ghi tay.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>Sheet Triệu chứng: xếp chip trên màn hình + cột 'Khách hay nói' để nhân viên gõ lời khách là ra chip đúng.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
           <t>Sheet Dấu hiệu nguy hiểm: danh sách nhân viên phải hỏi khách trước. Chấm 1 dấu hiệu là app không ra thuốc, chỉ bảo đi khám / gọi dược sĩ. Sửa theo ý dược sĩ.</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr"/>
-    </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>Cách app đổi mg ra gói / viên: mg cần uống ÷ mg của thuốc, làm tròn về ¼, ½, ¾, 1, 1½, 2... Siro: đổi ra ml theo mg/5 ml.</t>
-        </is>
-      </c>
+      <c r="A14" s="2" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
+          <t>Cách app đổi mg ra gói / viên: mg cần uống ÷ mg của thuốc, làm tròn về ¼, ½, ¾, 1, 1½, 2... Siro: đổi ra ml theo mg/5 ml.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
           <t>Chấm nhiều triệu chứng: cùng hoạt chất chỉ ra 1 dòng; cùng Nhóm thì lấy dòng Ưu tiên nhỏ nhất, dòng còn lại thành gợi ý 'hoặc'.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
-    </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
+      <c r="A17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>Dữ liệu trong file là VÍ DỤ tham khảo theo liều OTC thông dụng. Dược sĩ kiểm tra và chịu trách nhiệm trước khi dùng thật.</t>
         </is>
@@ -770,7 +782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:J61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -781,7 +793,8 @@
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="8" customWidth="1" min="8" max="8"/>
-    <col width="26" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="26" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
@@ -827,6 +840,11 @@
       </c>
       <c r="I1" s="5" t="inlineStr">
         <is>
+          <t>Vị trí</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
           <t>Ghi chú</t>
         </is>
       </c>
@@ -870,6 +888,11 @@
       <c r="H2" s="6" t="inlineStr"/>
       <c r="I2" s="6" t="inlineStr">
         <is>
+          <t>Kệ A1</t>
+        </is>
+      </c>
+      <c r="J2" s="6" t="inlineStr">
+        <is>
           <t>ghi chú tuỳ ý</t>
         </is>
       </c>
@@ -909,7 +932,12 @@
         </is>
       </c>
       <c r="H3" s="7" t="inlineStr"/>
-      <c r="I3" s="7" t="inlineStr"/>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>Kệ A1</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr"/>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="8" t="inlineStr">
@@ -946,7 +974,12 @@
         </is>
       </c>
       <c r="H4" s="8" t="inlineStr"/>
-      <c r="I4" s="8" t="inlineStr"/>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>Kệ A2</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr"/>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="7" t="inlineStr">
@@ -983,7 +1016,12 @@
         </is>
       </c>
       <c r="H5" s="7" t="inlineStr"/>
-      <c r="I5" s="7" t="inlineStr"/>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>Kệ A3</t>
+        </is>
+      </c>
+      <c r="J5" s="7" t="inlineStr"/>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="8" t="inlineStr">
@@ -1020,7 +1058,12 @@
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr"/>
-      <c r="I6" s="8" t="inlineStr"/>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>Kệ B1</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="inlineStr"/>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="7" t="inlineStr">
@@ -1057,7 +1100,12 @@
         </is>
       </c>
       <c r="H7" s="7" t="inlineStr"/>
-      <c r="I7" s="7" t="inlineStr"/>
+      <c r="I7" s="7" t="inlineStr">
+        <is>
+          <t>Kệ B2</t>
+        </is>
+      </c>
+      <c r="J7" s="7" t="inlineStr"/>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="8" t="inlineStr">
@@ -1096,6 +1144,11 @@
       <c r="H8" s="8" t="inlineStr"/>
       <c r="I8" s="8" t="inlineStr">
         <is>
+          <t>Kệ B3</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
+        <is>
           <t>bột sủi vị cam</t>
         </is>
       </c>
@@ -1135,7 +1188,12 @@
         </is>
       </c>
       <c r="H9" s="7" t="inlineStr"/>
-      <c r="I9" s="7" t="inlineStr"/>
+      <c r="I9" s="7" t="inlineStr">
+        <is>
+          <t>Kệ C1</t>
+        </is>
+      </c>
+      <c r="J9" s="7" t="inlineStr"/>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="8" t="inlineStr">
@@ -1172,7 +1230,12 @@
         </is>
       </c>
       <c r="H10" s="8" t="inlineStr"/>
-      <c r="I10" s="8" t="inlineStr"/>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>Kệ C2</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="inlineStr"/>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="7" t="inlineStr">
@@ -1213,6 +1276,11 @@
       <c r="H11" s="7" t="inlineStr"/>
       <c r="I11" s="7" t="inlineStr">
         <is>
+          <t>Tủ kính</t>
+        </is>
+      </c>
+      <c r="J11" s="7" t="inlineStr">
+        <is>
           <t>có caffein</t>
         </is>
       </c>
@@ -1252,7 +1320,12 @@
         </is>
       </c>
       <c r="H12" s="8" t="inlineStr"/>
-      <c r="I12" s="8" t="inlineStr"/>
+      <c r="I12" s="8" t="inlineStr">
+        <is>
+          <t>Ngăn kéo 1</t>
+        </is>
+      </c>
+      <c r="J12" s="8" t="inlineStr"/>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="7" t="inlineStr">
@@ -1289,7 +1362,12 @@
         </is>
       </c>
       <c r="H13" s="7" t="inlineStr"/>
-      <c r="I13" s="7" t="inlineStr"/>
+      <c r="I13" s="7" t="inlineStr">
+        <is>
+          <t>Ngăn kéo 2</t>
+        </is>
+      </c>
+      <c r="J13" s="7" t="inlineStr"/>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="8" t="inlineStr">
@@ -1328,6 +1406,11 @@
       <c r="H14" s="8" t="inlineStr"/>
       <c r="I14" s="8" t="inlineStr">
         <is>
+          <t>Kệ D1</t>
+        </is>
+      </c>
+      <c r="J14" s="8" t="inlineStr">
+        <is>
           <t>mg ghi theo 5 ml</t>
         </is>
       </c>
@@ -1367,7 +1450,12 @@
         </is>
       </c>
       <c r="H15" s="7" t="inlineStr"/>
-      <c r="I15" s="7" t="inlineStr"/>
+      <c r="I15" s="7" t="inlineStr">
+        <is>
+          <t>Kệ A1</t>
+        </is>
+      </c>
+      <c r="J15" s="7" t="inlineStr"/>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="8" t="inlineStr">
@@ -1404,7 +1492,12 @@
         </is>
       </c>
       <c r="H16" s="8" t="inlineStr"/>
-      <c r="I16" s="8" t="inlineStr"/>
+      <c r="I16" s="8" t="inlineStr">
+        <is>
+          <t>Kệ A2</t>
+        </is>
+      </c>
+      <c r="J16" s="8" t="inlineStr"/>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="7" t="inlineStr">
@@ -1441,7 +1534,12 @@
         </is>
       </c>
       <c r="H17" s="7" t="inlineStr"/>
-      <c r="I17" s="7" t="inlineStr"/>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>Kệ A3</t>
+        </is>
+      </c>
+      <c r="J17" s="7" t="inlineStr"/>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="8" t="inlineStr">
@@ -1478,7 +1576,12 @@
         </is>
       </c>
       <c r="H18" s="8" t="inlineStr"/>
-      <c r="I18" s="8" t="inlineStr"/>
+      <c r="I18" s="8" t="inlineStr">
+        <is>
+          <t>Kệ B1</t>
+        </is>
+      </c>
+      <c r="J18" s="8" t="inlineStr"/>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="7" t="inlineStr">
@@ -1517,6 +1620,11 @@
       <c r="H19" s="7" t="inlineStr"/>
       <c r="I19" s="7" t="inlineStr">
         <is>
+          <t>Kệ B2</t>
+        </is>
+      </c>
+      <c r="J19" s="7" t="inlineStr">
+        <is>
           <t>mg ghi theo 5 ml</t>
         </is>
       </c>
@@ -1556,7 +1664,12 @@
         </is>
       </c>
       <c r="H20" s="8" t="inlineStr"/>
-      <c r="I20" s="8" t="inlineStr"/>
+      <c r="I20" s="8" t="inlineStr">
+        <is>
+          <t>Kệ B3</t>
+        </is>
+      </c>
+      <c r="J20" s="8" t="inlineStr"/>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="7" t="inlineStr">
@@ -1595,6 +1708,11 @@
       <c r="H21" s="7" t="inlineStr"/>
       <c r="I21" s="7" t="inlineStr">
         <is>
+          <t>Kệ C1</t>
+        </is>
+      </c>
+      <c r="J21" s="7" t="inlineStr">
+        <is>
           <t>mg ghi theo 5 ml</t>
         </is>
       </c>
@@ -1634,7 +1752,12 @@
         </is>
       </c>
       <c r="H22" s="8" t="inlineStr"/>
-      <c r="I22" s="8" t="inlineStr"/>
+      <c r="I22" s="8" t="inlineStr">
+        <is>
+          <t>Kệ C2</t>
+        </is>
+      </c>
+      <c r="J22" s="8" t="inlineStr"/>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="7" t="inlineStr">
@@ -1671,6 +1794,11 @@
       <c r="H23" s="7" t="inlineStr"/>
       <c r="I23" s="7" t="inlineStr">
         <is>
+          <t>Tủ lạnh</t>
+        </is>
+      </c>
+      <c r="J23" s="7" t="inlineStr">
+        <is>
           <t>thảo dược, liều theo ml</t>
         </is>
       </c>
@@ -1712,6 +1840,11 @@
       <c r="H24" s="8" t="inlineStr"/>
       <c r="I24" s="8" t="inlineStr">
         <is>
+          <t>Ngăn kéo 1</t>
+        </is>
+      </c>
+      <c r="J24" s="8" t="inlineStr">
+        <is>
           <t>không buồn ngủ</t>
         </is>
       </c>
@@ -1751,7 +1884,12 @@
         </is>
       </c>
       <c r="H25" s="7" t="inlineStr"/>
-      <c r="I25" s="7" t="inlineStr"/>
+      <c r="I25" s="7" t="inlineStr">
+        <is>
+          <t>Ngăn kéo 2</t>
+        </is>
+      </c>
+      <c r="J25" s="7" t="inlineStr"/>
     </row>
     <row r="26" ht="22" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
@@ -1790,6 +1928,11 @@
       <c r="H26" s="8" t="inlineStr"/>
       <c r="I26" s="8" t="inlineStr">
         <is>
+          <t>Kệ D2</t>
+        </is>
+      </c>
+      <c r="J26" s="8" t="inlineStr">
+        <is>
           <t>mg ghi theo 5 ml</t>
         </is>
       </c>
@@ -1829,7 +1972,12 @@
         </is>
       </c>
       <c r="H27" s="7" t="inlineStr"/>
-      <c r="I27" s="7" t="inlineStr"/>
+      <c r="I27" s="7" t="inlineStr">
+        <is>
+          <t>Kệ A1</t>
+        </is>
+      </c>
+      <c r="J27" s="7" t="inlineStr"/>
     </row>
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="8" t="inlineStr">
@@ -1866,7 +2014,12 @@
         </is>
       </c>
       <c r="H28" s="8" t="inlineStr"/>
-      <c r="I28" s="8" t="inlineStr"/>
+      <c r="I28" s="8" t="inlineStr">
+        <is>
+          <t>Kệ A2</t>
+        </is>
+      </c>
+      <c r="J28" s="8" t="inlineStr"/>
     </row>
     <row r="29" ht="22" customHeight="1">
       <c r="A29" s="7" t="inlineStr">
@@ -1905,6 +2058,11 @@
       <c r="H29" s="7" t="inlineStr"/>
       <c r="I29" s="7" t="inlineStr">
         <is>
+          <t>Kệ A3</t>
+        </is>
+      </c>
+      <c r="J29" s="7" t="inlineStr">
+        <is>
           <t>gây buồn ngủ</t>
         </is>
       </c>
@@ -1944,7 +2102,12 @@
         </is>
       </c>
       <c r="H30" s="8" t="inlineStr"/>
-      <c r="I30" s="8" t="inlineStr"/>
+      <c r="I30" s="8" t="inlineStr">
+        <is>
+          <t>Kệ B1</t>
+        </is>
+      </c>
+      <c r="J30" s="8" t="inlineStr"/>
     </row>
     <row r="31" ht="22" customHeight="1">
       <c r="A31" s="7" t="inlineStr">
@@ -1981,7 +2144,12 @@
         </is>
       </c>
       <c r="H31" s="7" t="inlineStr"/>
-      <c r="I31" s="7" t="inlineStr"/>
+      <c r="I31" s="7" t="inlineStr">
+        <is>
+          <t>Kệ B2</t>
+        </is>
+      </c>
+      <c r="J31" s="7" t="inlineStr"/>
     </row>
     <row r="32" ht="22" customHeight="1">
       <c r="A32" s="8" t="inlineStr">
@@ -2020,6 +2188,11 @@
       <c r="H32" s="8" t="inlineStr"/>
       <c r="I32" s="8" t="inlineStr">
         <is>
+          <t>Kệ B3</t>
+        </is>
+      </c>
+      <c r="J32" s="8" t="inlineStr">
+        <is>
           <t>ngậm dưới lưỡi</t>
         </is>
       </c>
@@ -2059,6 +2232,11 @@
       <c r="H33" s="7" t="inlineStr"/>
       <c r="I33" s="7" t="inlineStr">
         <is>
+          <t>Kệ C1</t>
+        </is>
+      </c>
+      <c r="J33" s="7" t="inlineStr">
+        <is>
           <t>trên 6 tuổi</t>
         </is>
       </c>
@@ -2096,7 +2274,12 @@
         </is>
       </c>
       <c r="H34" s="8" t="inlineStr"/>
-      <c r="I34" s="8" t="inlineStr"/>
+      <c r="I34" s="8" t="inlineStr">
+        <is>
+          <t>Kệ C2</t>
+        </is>
+      </c>
+      <c r="J34" s="8" t="inlineStr"/>
     </row>
     <row r="35" ht="22" customHeight="1">
       <c r="A35" s="7" t="inlineStr">
@@ -2133,6 +2316,11 @@
       <c r="H35" s="7" t="inlineStr"/>
       <c r="I35" s="7" t="inlineStr">
         <is>
+          <t>Tủ kính</t>
+        </is>
+      </c>
+      <c r="J35" s="7" t="inlineStr">
+        <is>
           <t>nhỏ mũi, súc miệng</t>
         </is>
       </c>
@@ -2172,6 +2360,11 @@
       <c r="H36" s="8" t="inlineStr"/>
       <c r="I36" s="8" t="inlineStr">
         <is>
+          <t>Ngăn kéo 1</t>
+        </is>
+      </c>
+      <c r="J36" s="8" t="inlineStr">
+        <is>
           <t>không quá 5 ngày</t>
         </is>
       </c>
@@ -2211,6 +2404,11 @@
       <c r="H37" s="7" t="inlineStr"/>
       <c r="I37" s="7" t="inlineStr">
         <is>
+          <t>Ngăn kéo 2</t>
+        </is>
+      </c>
+      <c r="J37" s="7" t="inlineStr">
+        <is>
           <t>trên 6 tuổi</t>
         </is>
       </c>
@@ -2250,6 +2448,11 @@
       <c r="H38" s="8" t="inlineStr"/>
       <c r="I38" s="8" t="inlineStr">
         <is>
+          <t>Kệ D3</t>
+        </is>
+      </c>
+      <c r="J38" s="8" t="inlineStr">
+        <is>
           <t>pha đúng lượng nước</t>
         </is>
       </c>
@@ -2291,6 +2494,11 @@
       <c r="H39" s="7" t="inlineStr"/>
       <c r="I39" s="7" t="inlineStr">
         <is>
+          <t>Kệ A1</t>
+        </is>
+      </c>
+      <c r="J39" s="7" t="inlineStr">
+        <is>
           <t>gói 3 g</t>
         </is>
       </c>
@@ -2330,7 +2538,12 @@
         </is>
       </c>
       <c r="H40" s="8" t="inlineStr"/>
-      <c r="I40" s="8" t="inlineStr"/>
+      <c r="I40" s="8" t="inlineStr">
+        <is>
+          <t>Kệ A2</t>
+        </is>
+      </c>
+      <c r="J40" s="8" t="inlineStr"/>
     </row>
     <row r="41" ht="22" customHeight="1">
       <c r="A41" s="7" t="inlineStr">
@@ -2367,7 +2580,12 @@
         </is>
       </c>
       <c r="H41" s="7" t="inlineStr"/>
-      <c r="I41" s="7" t="inlineStr"/>
+      <c r="I41" s="7" t="inlineStr">
+        <is>
+          <t>Kệ A3</t>
+        </is>
+      </c>
+      <c r="J41" s="7" t="inlineStr"/>
     </row>
     <row r="42" ht="22" customHeight="1">
       <c r="A42" s="8" t="inlineStr">
@@ -2404,7 +2622,12 @@
         </is>
       </c>
       <c r="H42" s="8" t="inlineStr"/>
-      <c r="I42" s="8" t="inlineStr"/>
+      <c r="I42" s="8" t="inlineStr">
+        <is>
+          <t>Kệ B1</t>
+        </is>
+      </c>
+      <c r="J42" s="8" t="inlineStr"/>
     </row>
     <row r="43" ht="22" customHeight="1">
       <c r="A43" s="7" t="inlineStr">
@@ -2443,6 +2666,11 @@
       <c r="H43" s="7" t="inlineStr"/>
       <c r="I43" s="7" t="inlineStr">
         <is>
+          <t>Kệ B2</t>
+        </is>
+      </c>
+      <c r="J43" s="7" t="inlineStr">
+        <is>
           <t>không dùng trẻ dưới 12 tuổi</t>
         </is>
       </c>
@@ -2482,6 +2710,11 @@
       <c r="H44" s="8" t="inlineStr"/>
       <c r="I44" s="8" t="inlineStr">
         <is>
+          <t>Kệ B3</t>
+        </is>
+      </c>
+      <c r="J44" s="8" t="inlineStr">
+        <is>
           <t>men vi sinh</t>
         </is>
       </c>
@@ -2521,7 +2754,12 @@
         </is>
       </c>
       <c r="H45" s="7" t="inlineStr"/>
-      <c r="I45" s="7" t="inlineStr"/>
+      <c r="I45" s="7" t="inlineStr">
+        <is>
+          <t>Kệ C1</t>
+        </is>
+      </c>
+      <c r="J45" s="7" t="inlineStr"/>
     </row>
     <row r="46" ht="22" customHeight="1">
       <c r="A46" s="8" t="inlineStr">
@@ -2558,7 +2796,12 @@
         </is>
       </c>
       <c r="H46" s="8" t="inlineStr"/>
-      <c r="I46" s="8" t="inlineStr"/>
+      <c r="I46" s="8" t="inlineStr">
+        <is>
+          <t>Kệ C2</t>
+        </is>
+      </c>
+      <c r="J46" s="8" t="inlineStr"/>
     </row>
     <row r="47" ht="22" customHeight="1">
       <c r="A47" s="7" t="inlineStr">
@@ -2597,6 +2840,11 @@
       <c r="H47" s="7" t="inlineStr"/>
       <c r="I47" s="7" t="inlineStr">
         <is>
+          <t>Tủ kính</t>
+        </is>
+      </c>
+      <c r="J47" s="7" t="inlineStr">
+        <is>
           <t>uống trước ăn sáng</t>
         </is>
       </c>
@@ -2634,7 +2882,12 @@
         </is>
       </c>
       <c r="H48" s="8" t="inlineStr"/>
-      <c r="I48" s="8" t="inlineStr"/>
+      <c r="I48" s="8" t="inlineStr">
+        <is>
+          <t>Ngăn kéo 1</t>
+        </is>
+      </c>
+      <c r="J48" s="8" t="inlineStr"/>
     </row>
     <row r="49" ht="22" customHeight="1">
       <c r="A49" s="7" t="inlineStr">
@@ -2671,7 +2924,12 @@
         </is>
       </c>
       <c r="H49" s="7" t="inlineStr"/>
-      <c r="I49" s="7" t="inlineStr"/>
+      <c r="I49" s="7" t="inlineStr">
+        <is>
+          <t>Ngăn kéo 2</t>
+        </is>
+      </c>
+      <c r="J49" s="7" t="inlineStr"/>
     </row>
     <row r="50" ht="22" customHeight="1">
       <c r="A50" s="8" t="inlineStr">
@@ -2708,7 +2966,12 @@
         </is>
       </c>
       <c r="H50" s="8" t="inlineStr"/>
-      <c r="I50" s="8" t="inlineStr"/>
+      <c r="I50" s="8" t="inlineStr">
+        <is>
+          <t>Kệ D1</t>
+        </is>
+      </c>
+      <c r="J50" s="8" t="inlineStr"/>
     </row>
     <row r="51" ht="22" customHeight="1">
       <c r="A51" s="7" t="inlineStr">
@@ -2745,6 +3008,11 @@
       <c r="H51" s="7" t="inlineStr"/>
       <c r="I51" s="7" t="inlineStr">
         <is>
+          <t>Kệ A1</t>
+        </is>
+      </c>
+      <c r="J51" s="7" t="inlineStr">
+        <is>
           <t>10 g/15 ml</t>
         </is>
       </c>
@@ -2784,7 +3052,12 @@
         </is>
       </c>
       <c r="H52" s="8" t="inlineStr"/>
-      <c r="I52" s="8" t="inlineStr"/>
+      <c r="I52" s="8" t="inlineStr">
+        <is>
+          <t>Kệ A2</t>
+        </is>
+      </c>
+      <c r="J52" s="8" t="inlineStr"/>
     </row>
     <row r="53" ht="22" customHeight="1">
       <c r="A53" s="7" t="inlineStr">
@@ -2821,7 +3094,12 @@
         </is>
       </c>
       <c r="H53" s="7" t="inlineStr"/>
-      <c r="I53" s="7" t="inlineStr"/>
+      <c r="I53" s="7" t="inlineStr">
+        <is>
+          <t>Kệ A3</t>
+        </is>
+      </c>
+      <c r="J53" s="7" t="inlineStr"/>
     </row>
     <row r="54" ht="22" customHeight="1">
       <c r="A54" s="8" t="inlineStr">
@@ -2858,7 +3136,12 @@
         </is>
       </c>
       <c r="H54" s="8" t="inlineStr"/>
-      <c r="I54" s="8" t="inlineStr"/>
+      <c r="I54" s="8" t="inlineStr">
+        <is>
+          <t>Kệ B1</t>
+        </is>
+      </c>
+      <c r="J54" s="8" t="inlineStr"/>
     </row>
     <row r="55" ht="22" customHeight="1">
       <c r="A55" s="7" t="inlineStr">
@@ -2895,7 +3178,12 @@
         </is>
       </c>
       <c r="H55" s="7" t="inlineStr"/>
-      <c r="I55" s="7" t="inlineStr"/>
+      <c r="I55" s="7" t="inlineStr">
+        <is>
+          <t>Kệ B2</t>
+        </is>
+      </c>
+      <c r="J55" s="7" t="inlineStr"/>
     </row>
     <row r="56" ht="22" customHeight="1">
       <c r="A56" s="8" t="inlineStr">
@@ -2930,7 +3218,12 @@
         </is>
       </c>
       <c r="H56" s="8" t="inlineStr"/>
-      <c r="I56" s="8" t="inlineStr"/>
+      <c r="I56" s="8" t="inlineStr">
+        <is>
+          <t>Kệ B3</t>
+        </is>
+      </c>
+      <c r="J56" s="8" t="inlineStr"/>
     </row>
     <row r="57" ht="22" customHeight="1">
       <c r="A57" s="7" t="inlineStr">
@@ -2967,6 +3260,11 @@
       <c r="H57" s="7" t="inlineStr"/>
       <c r="I57" s="7" t="inlineStr">
         <is>
+          <t>Kệ C1</t>
+        </is>
+      </c>
+      <c r="J57" s="7" t="inlineStr">
+        <is>
           <t>bôi ngoài</t>
         </is>
       </c>
@@ -3010,6 +3308,11 @@
       <c r="H58" s="8" t="inlineStr"/>
       <c r="I58" s="8" t="inlineStr">
         <is>
+          <t>Kệ C2</t>
+        </is>
+      </c>
+      <c r="J58" s="8" t="inlineStr">
+        <is>
           <t>khách hay hỏi</t>
         </is>
       </c>
@@ -3053,6 +3356,11 @@
       <c r="H59" s="7" t="inlineStr"/>
       <c r="I59" s="7" t="inlineStr">
         <is>
+          <t>Tủ kính</t>
+        </is>
+      </c>
+      <c r="J59" s="7" t="inlineStr">
+        <is>
           <t>cảm cúm</t>
         </is>
       </c>
@@ -3094,7 +3402,12 @@
         </is>
       </c>
       <c r="H60" s="8" t="inlineStr"/>
-      <c r="I60" s="8" t="inlineStr"/>
+      <c r="I60" s="8" t="inlineStr">
+        <is>
+          <t>Ngăn kéo 1</t>
+        </is>
+      </c>
+      <c r="J60" s="8" t="inlineStr"/>
     </row>
     <row r="61" ht="22" customHeight="1">
       <c r="A61" s="7" t="inlineStr">
@@ -3139,25 +3452,30 @@
       </c>
       <c r="I61" s="7" t="inlineStr">
         <is>
+          <t>Ngăn kéo 2</t>
+        </is>
+      </c>
+      <c r="J61" s="7" t="inlineStr">
+        <is>
           <t>kháng sinh, phải có toa</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I61"/>
+  <autoFilter ref="A1:J61"/>
   <conditionalFormatting sqref="A3:A361">
     <cfRule type="expression" priority="1" dxfId="0">
-      <formula>AND(COUNTA($A3:$I3)&gt;0,A3="")</formula>
+      <formula>AND(COUNTA($A3:$J3)&gt;0,A3="")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B3:B361">
     <cfRule type="expression" priority="2" dxfId="0">
-      <formula>AND(COUNTA($A3:$I3)&gt;0,B3="")</formula>
+      <formula>AND(COUNTA($A3:$J3)&gt;0,B3="")</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D3:D361">
     <cfRule type="expression" priority="3" dxfId="0">
-      <formula>AND(COUNTA($A3:$I3)&gt;0,D3="")</formula>
+      <formula>AND(COUNTA($A3:$J3)&gt;0,D3="")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="4">

</xml_diff>